<commit_message>
feat: add deterministic synthetic evaluation corpus
</commit_message>
<xml_diff>
--- a/examples/corpus/demo/inventory/inventario-procesos.xlsx
+++ b/examples/corpus/demo/inventory/inventario-procesos.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procesos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contactos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,21 +418,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proceso</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>SLA</t>
         </is>
@@ -464,6 +474,77 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>Lunes 06:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PUB_CLIENTES_21</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Calidad de Datos</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Buzón sintético</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DataOps</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>dataops@example.invalid</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Backoffice</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>backoffice@example.invalid</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WRK-TASK-026: corpus y gold sets sintéticos (#5)
* feat: add deterministic synthetic evaluation corpus

* docs: complete WRK-TASK-026 evidence
</commit_message>
<xml_diff>
--- a/examples/corpus/demo/inventory/inventario-procesos.xlsx
+++ b/examples/corpus/demo/inventory/inventario-procesos.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procesos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contactos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,21 +418,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proceso</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>SLA</t>
         </is>
@@ -464,6 +474,77 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>Lunes 06:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PUB_CLIENTES_21</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Calidad de Datos</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Buzón sintético</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DataOps</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>dataops@example.invalid</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Backoffice</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>backoffice@example.invalid</t>
         </is>
       </c>
     </row>

</xml_diff>